<commit_message>
Add site scorecard, coding review and lock readiness from EDC reports
- rtcrcore: query_status(), form_status(), entry_lag(), site_scorecard(),
  lock_readiness(), lock_by_subject() and coding_review(), all derived
  against the review date; new "report" form type for operational EDC
  reports, kept out of clinical screens
- rtcrapp: site scorecard, coding review and lock readiness modules;
  listings show unresolved queries per record
- Example study: simulated query and form status reports and MedDRA
  version on AE coding (dev/simulate_example_ops.R), mapped in the spec
- Fix: timeline clicks did not open the subject profile (navigation used
  the module's session) and plotly logged a warning on every flush
- README and design doc updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/studies/example/mapping_spec.xlsx
+++ b/studies/example/mapping_spec.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="190">
   <si>
     <t xml:space="preserve">FORMOID</t>
   </si>
@@ -488,6 +488,102 @@
   </si>
   <si>
     <t xml:space="preserve">VERY MUCH IMPROVED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUERY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edc_queries.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDC query report; available from the open date, status derived from the dates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSTAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edc_formstatus.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUBJID, FOLDER, FORM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDC form status: SDV, PI signature, freeze and lock dates per form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEDDRAV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MedDRA version of the code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPENDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Query exists from the day it is opened</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYFORM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FORM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form of the queried record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Record key for log forms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYTEXT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYSTAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYSTATUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status on the extract date; the review date status is derived from the dates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYOPDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYANSDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANSWERDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRYCLSDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLOSEDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form status exists from the day the form is entered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSFORM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDVDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIGNDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FREEZEDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOCKDT</t>
   </si>
 </sst>
 </file>
@@ -1036,6 +1132,46 @@
         <v>43</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>163</v>
+      </c>
+      <c r="B12" t="s">
+        <v>159</v>
+      </c>
+      <c r="C12" t="s">
+        <v>164</v>
+      </c>
+      <c r="D12" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>166</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2382,22 +2518,20 @@
         <v>26</v>
       </c>
       <c r="B65" t="s">
-        <v>102</v>
+        <v>167</v>
       </c>
       <c r="C65" t="s">
-        <v>102</v>
+        <v>167</v>
       </c>
       <c r="D65" t="s">
-        <v>59</v>
-      </c>
-      <c r="E65" t="s">
-        <v>103</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E65"/>
       <c r="F65" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="G65" t="s">
-        <v>104</v>
+        <v>168</v>
       </c>
     </row>
     <row r="66">
@@ -2405,29 +2539,33 @@
         <v>26</v>
       </c>
       <c r="B66" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C66" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D66" t="s">
-        <v>54</v>
-      </c>
-      <c r="E66"/>
+        <v>59</v>
+      </c>
+      <c r="E66" t="s">
+        <v>103</v>
+      </c>
       <c r="F66" t="s">
         <v>55</v>
       </c>
-      <c r="G66"/>
+      <c r="G66" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
         <v>26</v>
       </c>
       <c r="B67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D67" t="s">
         <v>54</v>
@@ -2443,10 +2581,10 @@
         <v>26</v>
       </c>
       <c r="B68" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C68" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D68" t="s">
         <v>54</v>
@@ -2462,10 +2600,10 @@
         <v>26</v>
       </c>
       <c r="B69" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C69" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D69" t="s">
         <v>54</v>
@@ -2478,13 +2616,13 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B70" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="C70" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="D70" t="s">
         <v>54</v>
@@ -2500,10 +2638,10 @@
         <v>31</v>
       </c>
       <c r="B71" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C71" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D71" t="s">
         <v>54</v>
@@ -2519,10 +2657,10 @@
         <v>31</v>
       </c>
       <c r="B72" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C72" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="D72" t="s">
         <v>54</v>
@@ -2538,10 +2676,10 @@
         <v>31</v>
       </c>
       <c r="B73" t="s">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="C73" t="s">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="D73" t="s">
         <v>54</v>
@@ -2557,17 +2695,15 @@
         <v>31</v>
       </c>
       <c r="B74" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C74" t="s">
         <v>75</v>
       </c>
       <c r="D74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E74" t="s">
-        <v>77</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E74"/>
       <c r="F74" t="s">
         <v>55</v>
       </c>
@@ -2578,33 +2714,31 @@
         <v>31</v>
       </c>
       <c r="B75" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="C75" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D75" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E75" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F75" t="s">
         <v>55</v>
       </c>
-      <c r="G75" t="s">
-        <v>61</v>
-      </c>
+      <c r="G75"/>
     </row>
     <row r="76">
       <c r="A76" t="s">
         <v>31</v>
       </c>
       <c r="B76" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C76" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D76" t="s">
         <v>59</v>
@@ -2616,7 +2750,7 @@
         <v>55</v>
       </c>
       <c r="G76" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="77">
@@ -2624,7 +2758,7 @@
         <v>31</v>
       </c>
       <c r="B77" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C77" t="s">
         <v>63</v>
@@ -2633,13 +2767,13 @@
         <v>59</v>
       </c>
       <c r="E77" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F77" t="s">
         <v>55</v>
       </c>
       <c r="G77" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="78">
@@ -2647,31 +2781,33 @@
         <v>31</v>
       </c>
       <c r="B78" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="C78" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="D78" t="s">
         <v>59</v>
       </c>
       <c r="E78" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="F78" t="s">
         <v>55</v>
       </c>
-      <c r="G78"/>
+      <c r="G78" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
         <v>31</v>
       </c>
       <c r="B79" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C79" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D79" t="s">
         <v>59</v>
@@ -2689,15 +2825,17 @@
         <v>31</v>
       </c>
       <c r="B80" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C80" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D80" t="s">
-        <v>69</v>
-      </c>
-      <c r="E80"/>
+        <v>59</v>
+      </c>
+      <c r="E80" t="s">
+        <v>74</v>
+      </c>
       <c r="F80" t="s">
         <v>55</v>
       </c>
@@ -2708,10 +2846,10 @@
         <v>31</v>
       </c>
       <c r="B81" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C81" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D81" t="s">
         <v>69</v>
@@ -2724,16 +2862,16 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B82" t="s">
-        <v>53</v>
+        <v>112</v>
       </c>
       <c r="C82" t="s">
-        <v>53</v>
+        <v>112</v>
       </c>
       <c r="D82" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E82"/>
       <c r="F82" t="s">
@@ -2746,52 +2884,52 @@
         <v>34</v>
       </c>
       <c r="B83" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C83" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="D83" t="s">
-        <v>113</v>
-      </c>
-      <c r="E83" t="s">
-        <v>114</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E83"/>
       <c r="F83" t="s">
         <v>55</v>
       </c>
-      <c r="G83" t="s">
-        <v>115</v>
-      </c>
+      <c r="G83"/>
     </row>
     <row r="84">
       <c r="A84" t="s">
         <v>34</v>
       </c>
       <c r="B84" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C84" t="s">
         <v>9</v>
       </c>
       <c r="D84" t="s">
-        <v>54</v>
-      </c>
-      <c r="E84"/>
+        <v>113</v>
+      </c>
+      <c r="E84" t="s">
+        <v>114</v>
+      </c>
       <c r="F84" t="s">
         <v>55</v>
       </c>
-      <c r="G84"/>
+      <c r="G84" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
         <v>34</v>
       </c>
       <c r="B85" t="s">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="C85" t="s">
-        <v>116</v>
+        <v>9</v>
       </c>
       <c r="D85" t="s">
         <v>54</v>
@@ -2800,60 +2938,56 @@
       <c r="F85" t="s">
         <v>55</v>
       </c>
-      <c r="G85" t="s">
-        <v>117</v>
-      </c>
+      <c r="G85"/>
     </row>
     <row r="86">
       <c r="A86" t="s">
         <v>34</v>
       </c>
       <c r="B86" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C86" t="s">
         <v>116</v>
       </c>
       <c r="D86" t="s">
-        <v>13</v>
-      </c>
-      <c r="E86" t="s">
-        <v>118</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E86"/>
       <c r="F86" t="s">
         <v>55</v>
       </c>
-      <c r="G86"/>
+      <c r="G86" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
         <v>34</v>
       </c>
       <c r="B87" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="C87" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D87" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E87" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F87" t="s">
         <v>55</v>
       </c>
-      <c r="G87" t="s">
-        <v>121</v>
-      </c>
+      <c r="G87"/>
     </row>
     <row r="88">
       <c r="A88" t="s">
         <v>34</v>
       </c>
       <c r="B88" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C88" t="s">
         <v>119</v>
@@ -2862,7 +2996,7 @@
         <v>59</v>
       </c>
       <c r="E88" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F88" t="s">
         <v>55</v>
@@ -2876,38 +3010,42 @@
         <v>34</v>
       </c>
       <c r="B89" t="s">
-        <v>123</v>
+        <v>65</v>
       </c>
       <c r="C89" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D89" t="s">
         <v>59</v>
       </c>
       <c r="E89" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F89" t="s">
         <v>55</v>
       </c>
-      <c r="G89"/>
+      <c r="G89" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
         <v>34</v>
       </c>
       <c r="B90" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C90" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D90" t="s">
-        <v>54</v>
-      </c>
-      <c r="E90"/>
+        <v>59</v>
+      </c>
+      <c r="E90" t="s">
+        <v>120</v>
+      </c>
       <c r="F90" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="G90"/>
     </row>
@@ -2916,17 +3054,15 @@
         <v>34</v>
       </c>
       <c r="B91" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C91" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D91" t="s">
-        <v>59</v>
-      </c>
-      <c r="E91" t="s">
-        <v>120</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E91"/>
       <c r="F91" t="s">
         <v>71</v>
       </c>
@@ -2937,17 +3073,19 @@
         <v>34</v>
       </c>
       <c r="B92" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="C92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D92" t="s">
-        <v>69</v>
-      </c>
-      <c r="E92"/>
+        <v>59</v>
+      </c>
+      <c r="E92" t="s">
+        <v>120</v>
+      </c>
       <c r="F92" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="G92"/>
     </row>
@@ -2956,31 +3094,29 @@
         <v>34</v>
       </c>
       <c r="B93" t="s">
-        <v>127</v>
+        <v>34</v>
       </c>
       <c r="C93" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D93" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E93"/>
       <c r="F93" t="s">
         <v>55</v>
       </c>
-      <c r="G93" t="s">
-        <v>129</v>
-      </c>
+      <c r="G93"/>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B94" t="s">
-        <v>53</v>
+        <v>127</v>
       </c>
       <c r="C94" t="s">
-        <v>53</v>
+        <v>128</v>
       </c>
       <c r="D94" t="s">
         <v>54</v>
@@ -2989,59 +3125,61 @@
       <c r="F94" t="s">
         <v>55</v>
       </c>
-      <c r="G94"/>
+      <c r="G94" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
         <v>40</v>
       </c>
       <c r="B95" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C95" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="D95" t="s">
-        <v>113</v>
-      </c>
-      <c r="E95" t="s">
-        <v>114</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E95"/>
       <c r="F95" t="s">
         <v>55</v>
       </c>
-      <c r="G95" t="s">
-        <v>115</v>
-      </c>
+      <c r="G95"/>
     </row>
     <row r="96">
       <c r="A96" t="s">
         <v>40</v>
       </c>
       <c r="B96" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C96" t="s">
         <v>9</v>
       </c>
       <c r="D96" t="s">
-        <v>54</v>
-      </c>
-      <c r="E96"/>
+        <v>113</v>
+      </c>
+      <c r="E96" t="s">
+        <v>114</v>
+      </c>
       <c r="F96" t="s">
         <v>55</v>
       </c>
-      <c r="G96"/>
+      <c r="G96" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
         <v>40</v>
       </c>
       <c r="B97" t="s">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="C97" t="s">
-        <v>116</v>
+        <v>9</v>
       </c>
       <c r="D97" t="s">
         <v>54</v>
@@ -3050,60 +3188,56 @@
       <c r="F97" t="s">
         <v>55</v>
       </c>
-      <c r="G97" t="s">
-        <v>117</v>
-      </c>
+      <c r="G97"/>
     </row>
     <row r="98">
       <c r="A98" t="s">
         <v>40</v>
       </c>
       <c r="B98" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C98" t="s">
         <v>116</v>
       </c>
       <c r="D98" t="s">
-        <v>13</v>
-      </c>
-      <c r="E98" t="s">
-        <v>118</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E98"/>
       <c r="F98" t="s">
         <v>55</v>
       </c>
-      <c r="G98"/>
+      <c r="G98" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
         <v>40</v>
       </c>
       <c r="B99" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="C99" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D99" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E99" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F99" t="s">
         <v>55</v>
       </c>
-      <c r="G99" t="s">
-        <v>121</v>
-      </c>
+      <c r="G99"/>
     </row>
     <row r="100">
       <c r="A100" t="s">
         <v>40</v>
       </c>
       <c r="B100" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C100" t="s">
         <v>119</v>
@@ -3112,7 +3246,7 @@
         <v>59</v>
       </c>
       <c r="E100" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F100" t="s">
         <v>55</v>
@@ -3126,22 +3260,22 @@
         <v>40</v>
       </c>
       <c r="B101" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C101" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D101" t="s">
         <v>59</v>
       </c>
       <c r="E101" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F101" t="s">
         <v>55</v>
       </c>
       <c r="G101" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="102">
@@ -3149,36 +3283,40 @@
         <v>40</v>
       </c>
       <c r="B102" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C102" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D102" t="s">
-        <v>54</v>
-      </c>
-      <c r="E102"/>
+        <v>59</v>
+      </c>
+      <c r="E102" t="s">
+        <v>131</v>
+      </c>
       <c r="F102" t="s">
         <v>55</v>
       </c>
-      <c r="G102"/>
+      <c r="G102" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
         <v>40</v>
       </c>
       <c r="B103" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C103" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D103" t="s">
         <v>54</v>
       </c>
       <c r="E103"/>
       <c r="F103" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="G103"/>
     </row>
@@ -3187,17 +3325,17 @@
         <v>40</v>
       </c>
       <c r="B104" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C104" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D104" t="s">
         <v>54</v>
       </c>
       <c r="E104"/>
       <c r="F104" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="G104"/>
     </row>
@@ -3206,61 +3344,589 @@
         <v>40</v>
       </c>
       <c r="B105" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C105" t="s">
         <v>135</v>
       </c>
       <c r="D105" t="s">
-        <v>69</v>
-      </c>
-      <c r="E105" t="s">
-        <v>137</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="E105"/>
       <c r="F105" t="s">
         <v>55</v>
       </c>
-      <c r="G105" t="s">
-        <v>138</v>
-      </c>
+      <c r="G105"/>
     </row>
     <row r="106">
       <c r="A106" t="s">
         <v>40</v>
       </c>
       <c r="B106" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C106" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D106" t="s">
-        <v>54</v>
-      </c>
-      <c r="E106"/>
+        <v>69</v>
+      </c>
+      <c r="E106" t="s">
+        <v>137</v>
+      </c>
       <c r="F106" t="s">
         <v>55</v>
       </c>
-      <c r="G106"/>
+      <c r="G106" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
         <v>40</v>
       </c>
       <c r="B107" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C107" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D107" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="E107"/>
       <c r="F107" t="s">
         <v>55</v>
       </c>
       <c r="G107"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>40</v>
+      </c>
+      <c r="B108" t="s">
+        <v>140</v>
+      </c>
+      <c r="C108" t="s">
+        <v>140</v>
+      </c>
+      <c r="D108" t="s">
+        <v>69</v>
+      </c>
+      <c r="E108"/>
+      <c r="F108" t="s">
+        <v>55</v>
+      </c>
+      <c r="G108"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>158</v>
+      </c>
+      <c r="B109" t="s">
+        <v>53</v>
+      </c>
+      <c r="C109" t="s">
+        <v>53</v>
+      </c>
+      <c r="D109" t="s">
+        <v>54</v>
+      </c>
+      <c r="E109"/>
+      <c r="F109" t="s">
+        <v>55</v>
+      </c>
+      <c r="G109"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>158</v>
+      </c>
+      <c r="B110" t="s">
+        <v>56</v>
+      </c>
+      <c r="C110" t="s">
+        <v>56</v>
+      </c>
+      <c r="D110" t="s">
+        <v>54</v>
+      </c>
+      <c r="E110"/>
+      <c r="F110" t="s">
+        <v>55</v>
+      </c>
+      <c r="G110"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>158</v>
+      </c>
+      <c r="B111" t="s">
+        <v>9</v>
+      </c>
+      <c r="C111" t="s">
+        <v>9</v>
+      </c>
+      <c r="D111" t="s">
+        <v>54</v>
+      </c>
+      <c r="E111"/>
+      <c r="F111" t="s">
+        <v>55</v>
+      </c>
+      <c r="G111"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>158</v>
+      </c>
+      <c r="B112" t="s">
+        <v>75</v>
+      </c>
+      <c r="C112" t="s">
+        <v>75</v>
+      </c>
+      <c r="D112" t="s">
+        <v>54</v>
+      </c>
+      <c r="E112"/>
+      <c r="F112" t="s">
+        <v>55</v>
+      </c>
+      <c r="G112"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>158</v>
+      </c>
+      <c r="B113" t="s">
+        <v>57</v>
+      </c>
+      <c r="C113" t="s">
+        <v>169</v>
+      </c>
+      <c r="D113" t="s">
+        <v>59</v>
+      </c>
+      <c r="E113" t="s">
+        <v>60</v>
+      </c>
+      <c r="F113" t="s">
+        <v>55</v>
+      </c>
+      <c r="G113"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>158</v>
+      </c>
+      <c r="B114" t="s">
+        <v>65</v>
+      </c>
+      <c r="C114" t="s">
+        <v>169</v>
+      </c>
+      <c r="D114" t="s">
+        <v>59</v>
+      </c>
+      <c r="E114" t="s">
+        <v>66</v>
+      </c>
+      <c r="F114" t="s">
+        <v>55</v>
+      </c>
+      <c r="G114" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>158</v>
+      </c>
+      <c r="B115" t="s">
+        <v>171</v>
+      </c>
+      <c r="C115" t="s">
+        <v>172</v>
+      </c>
+      <c r="D115" t="s">
+        <v>54</v>
+      </c>
+      <c r="E115"/>
+      <c r="F115" t="s">
+        <v>55</v>
+      </c>
+      <c r="G115" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>158</v>
+      </c>
+      <c r="B116" t="s">
+        <v>95</v>
+      </c>
+      <c r="C116" t="s">
+        <v>95</v>
+      </c>
+      <c r="D116" t="s">
+        <v>54</v>
+      </c>
+      <c r="E116"/>
+      <c r="F116" t="s">
+        <v>71</v>
+      </c>
+      <c r="G116" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>158</v>
+      </c>
+      <c r="B117" t="s">
+        <v>175</v>
+      </c>
+      <c r="C117" t="s">
+        <v>175</v>
+      </c>
+      <c r="D117" t="s">
+        <v>54</v>
+      </c>
+      <c r="E117"/>
+      <c r="F117" t="s">
+        <v>55</v>
+      </c>
+      <c r="G117"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>158</v>
+      </c>
+      <c r="B118" t="s">
+        <v>176</v>
+      </c>
+      <c r="C118" t="s">
+        <v>177</v>
+      </c>
+      <c r="D118" t="s">
+        <v>54</v>
+      </c>
+      <c r="E118"/>
+      <c r="F118" t="s">
+        <v>55</v>
+      </c>
+      <c r="G118" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>158</v>
+      </c>
+      <c r="B119" t="s">
+        <v>179</v>
+      </c>
+      <c r="C119" t="s">
+        <v>169</v>
+      </c>
+      <c r="D119" t="s">
+        <v>59</v>
+      </c>
+      <c r="E119" t="s">
+        <v>60</v>
+      </c>
+      <c r="F119" t="s">
+        <v>55</v>
+      </c>
+      <c r="G119"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>158</v>
+      </c>
+      <c r="B120" t="s">
+        <v>180</v>
+      </c>
+      <c r="C120" t="s">
+        <v>181</v>
+      </c>
+      <c r="D120" t="s">
+        <v>59</v>
+      </c>
+      <c r="E120" t="s">
+        <v>60</v>
+      </c>
+      <c r="F120" t="s">
+        <v>55</v>
+      </c>
+      <c r="G120"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>158</v>
+      </c>
+      <c r="B121" t="s">
+        <v>182</v>
+      </c>
+      <c r="C121" t="s">
+        <v>183</v>
+      </c>
+      <c r="D121" t="s">
+        <v>59</v>
+      </c>
+      <c r="E121" t="s">
+        <v>60</v>
+      </c>
+      <c r="F121" t="s">
+        <v>55</v>
+      </c>
+      <c r="G121"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>163</v>
+      </c>
+      <c r="B122" t="s">
+        <v>53</v>
+      </c>
+      <c r="C122" t="s">
+        <v>53</v>
+      </c>
+      <c r="D122" t="s">
+        <v>54</v>
+      </c>
+      <c r="E122"/>
+      <c r="F122" t="s">
+        <v>55</v>
+      </c>
+      <c r="G122"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>163</v>
+      </c>
+      <c r="B123" t="s">
+        <v>56</v>
+      </c>
+      <c r="C123" t="s">
+        <v>56</v>
+      </c>
+      <c r="D123" t="s">
+        <v>54</v>
+      </c>
+      <c r="E123"/>
+      <c r="F123" t="s">
+        <v>55</v>
+      </c>
+      <c r="G123"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>163</v>
+      </c>
+      <c r="B124" t="s">
+        <v>9</v>
+      </c>
+      <c r="C124" t="s">
+        <v>9</v>
+      </c>
+      <c r="D124" t="s">
+        <v>54</v>
+      </c>
+      <c r="E124"/>
+      <c r="F124" t="s">
+        <v>55</v>
+      </c>
+      <c r="G124"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>163</v>
+      </c>
+      <c r="B125" t="s">
+        <v>75</v>
+      </c>
+      <c r="C125" t="s">
+        <v>75</v>
+      </c>
+      <c r="D125" t="s">
+        <v>54</v>
+      </c>
+      <c r="E125"/>
+      <c r="F125" t="s">
+        <v>55</v>
+      </c>
+      <c r="G125"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>163</v>
+      </c>
+      <c r="B126" t="s">
+        <v>57</v>
+      </c>
+      <c r="C126" t="s">
+        <v>58</v>
+      </c>
+      <c r="D126" t="s">
+        <v>59</v>
+      </c>
+      <c r="E126" t="s">
+        <v>60</v>
+      </c>
+      <c r="F126" t="s">
+        <v>55</v>
+      </c>
+      <c r="G126"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>163</v>
+      </c>
+      <c r="B127" t="s">
+        <v>65</v>
+      </c>
+      <c r="C127" t="s">
+        <v>58</v>
+      </c>
+      <c r="D127" t="s">
+        <v>59</v>
+      </c>
+      <c r="E127" t="s">
+        <v>66</v>
+      </c>
+      <c r="F127" t="s">
+        <v>55</v>
+      </c>
+      <c r="G127" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>163</v>
+      </c>
+      <c r="B128" t="s">
+        <v>62</v>
+      </c>
+      <c r="C128" t="s">
+        <v>63</v>
+      </c>
+      <c r="D128" t="s">
+        <v>59</v>
+      </c>
+      <c r="E128" t="s">
+        <v>60</v>
+      </c>
+      <c r="F128" t="s">
+        <v>55</v>
+      </c>
+      <c r="G128"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>163</v>
+      </c>
+      <c r="B129" t="s">
+        <v>185</v>
+      </c>
+      <c r="C129" t="s">
+        <v>172</v>
+      </c>
+      <c r="D129" t="s">
+        <v>54</v>
+      </c>
+      <c r="E129"/>
+      <c r="F129" t="s">
+        <v>55</v>
+      </c>
+      <c r="G129"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>163</v>
+      </c>
+      <c r="B130" t="s">
+        <v>186</v>
+      </c>
+      <c r="C130" t="s">
+        <v>186</v>
+      </c>
+      <c r="D130" t="s">
+        <v>59</v>
+      </c>
+      <c r="E130" t="s">
+        <v>74</v>
+      </c>
+      <c r="F130" t="s">
+        <v>55</v>
+      </c>
+      <c r="G130"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>163</v>
+      </c>
+      <c r="B131" t="s">
+        <v>187</v>
+      </c>
+      <c r="C131" t="s">
+        <v>187</v>
+      </c>
+      <c r="D131" t="s">
+        <v>59</v>
+      </c>
+      <c r="E131" t="s">
+        <v>74</v>
+      </c>
+      <c r="F131" t="s">
+        <v>55</v>
+      </c>
+      <c r="G131"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>163</v>
+      </c>
+      <c r="B132" t="s">
+        <v>188</v>
+      </c>
+      <c r="C132" t="s">
+        <v>188</v>
+      </c>
+      <c r="D132" t="s">
+        <v>59</v>
+      </c>
+      <c r="E132" t="s">
+        <v>74</v>
+      </c>
+      <c r="F132" t="s">
+        <v>55</v>
+      </c>
+      <c r="G132"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>163</v>
+      </c>
+      <c r="B133" t="s">
+        <v>189</v>
+      </c>
+      <c r="C133" t="s">
+        <v>189</v>
+      </c>
+      <c r="D133" t="s">
+        <v>59</v>
+      </c>
+      <c r="E133" t="s">
+        <v>74</v>
+      </c>
+      <c r="F133" t="s">
+        <v>55</v>
+      </c>
+      <c r="G133"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>

</xml_diff>